<commit_message>
updated code to show live LTP & added add New RM Option
</commit_message>
<xml_diff>
--- a/data/input/client_data.xlsx
+++ b/data/input/client_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="48">
   <si>
     <t>id</t>
   </si>
@@ -50,6 +50,114 @@
   </si>
   <si>
     <t>login_message</t>
+  </si>
+  <si>
+    <t>cc0f61ef-d534-49c4-b909-df4f0992989d</t>
+  </si>
+  <si>
+    <t>a3ea1d5a-0537-40b3-9145-3cc6603c3938</t>
+  </si>
+  <si>
+    <t>72e360b7-3528-4750-a7cc-80c9f6934a09</t>
+  </si>
+  <si>
+    <t>118db1ae-20d6-4f40-8351-3b48dcaf7184</t>
+  </si>
+  <si>
+    <t>ccf1b674-bd4a-4dba-903f-4e5125d35199</t>
+  </si>
+  <si>
+    <t>da21c621-85b6-42af-8b63-a420c080fa11</t>
+  </si>
+  <si>
+    <t>1ca9dc95-ca62-4825-8696-59b643315ea6</t>
+  </si>
+  <si>
+    <t>114</t>
+  </si>
+  <si>
+    <t>126</t>
+  </si>
+  <si>
+    <t>123445</t>
+  </si>
+  <si>
+    <t>11144</t>
+  </si>
+  <si>
+    <t>1744740</t>
+  </si>
+  <si>
+    <t>216199</t>
+  </si>
+  <si>
+    <t>233742</t>
+  </si>
+  <si>
+    <t>236901</t>
+  </si>
+  <si>
+    <t>243900</t>
+  </si>
+  <si>
+    <t>Thakur@123</t>
+  </si>
+  <si>
+    <t>manju@1234</t>
+  </si>
+  <si>
+    <t>TikaGautam@123</t>
+  </si>
+  <si>
+    <t>nepal123</t>
+  </si>
+  <si>
+    <t>Mahalaxmi6</t>
+  </si>
+  <si>
+    <t>Bhim@1234!</t>
+  </si>
+  <si>
+    <t>THAKUR</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>YUBARAJ</t>
+  </si>
+  <si>
+    <t>SAJAN</t>
+  </si>
+  <si>
+    <t>Ashwin Das</t>
+  </si>
+  <si>
+    <t>Manju Acharya Khanal</t>
+  </si>
+  <si>
+    <t>Tika Gautam</t>
+  </si>
+  <si>
+    <t>Ram Chandra Pokharel</t>
+  </si>
+  <si>
+    <t>Kuber Thapa</t>
+  </si>
+  <si>
+    <t>Laxman Limbu Subba</t>
+  </si>
+  <si>
+    <t>Bhim Prasad Sapkota</t>
+  </si>
+  <si>
+    <t>CRED</t>
+  </si>
+  <si>
+    <t>Failed: Username or password invalid.</t>
+  </si>
+  <si>
+    <t>Log in successful.</t>
   </si>
 </sst>
 </file>
@@ -407,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -446,6 +554,272 @@
       </c>
       <c r="L1" s="1" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+      <c r="K3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+      <c r="K4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" t="s">
+        <v>45</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K5" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" t="s">
+        <v>45</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K8" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>